<commit_message>
fix: MR commodity classification + debt mapping + rating PG compat
- vecm_bridge: pattern-based commodity detection (lme_*, steel_*, brent, etc.)
  LME Ni/Cu/Pd/Pt now properly classified as MR (was EWA fallback)
- orchestrator: forecast_years from project.yaml (was hardcoded 5)
- rating/runner: legacy rating_results wrapped in try/except for PG
- ExcelLoader: segments use repo.upsert_segment_data for PG compat
- Nornickel debt: fixed column mapping in template (was shifted)
- Nornickel template: db_unit=USD in meta (PG stores full USD)

Model results: LME MR forecasts (Ni $15.8k, Cu $9.1k→$8.4k, Pd $949→$919)
Rating: BBB+ → A- → A | BS_diff=$0 | 11 scenarios

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/companies/nornickel_v2/data/excel/nornickel_v2_template_v3.xlsx
+++ b/companies/nornickel_v2/data/excel/nornickel_v2_template_v3.xlsx
@@ -557,7 +557,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>mUSD</t>
+          <t>USD</t>
         </is>
       </c>
     </row>
@@ -10262,42 +10262,42 @@
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>opening_balance_mUSD</t>
+          <t>opening_balance_musd</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>committed_amount_mUSD</t>
+          <t>maturity_date</t>
         </is>
       </c>
       <c r="G1" s="5" t="inlineStr">
         <is>
-          <t>maturity_date</t>
+          <t>interest_rate</t>
         </is>
       </c>
       <c r="H1" s="5" t="inlineStr">
         <is>
-          <t>interest_rate</t>
+          <t>rate_type</t>
         </is>
       </c>
       <c r="I1" s="5" t="inlineStr">
         <is>
-          <t>rate_type</t>
+          <t>base_rate_factor</t>
         </is>
       </c>
       <c r="J1" s="5" t="inlineStr">
         <is>
-          <t>base_rate_factor</t>
+          <t>payment_frequency</t>
         </is>
       </c>
       <c r="K1" s="5" t="inlineStr">
         <is>
-          <t>payment_frequency</t>
+          <t>amortization_profile</t>
         </is>
       </c>
       <c r="L1" s="5" t="inlineStr">
         <is>
-          <t>amortization_profile</t>
+          <t>callable_flag</t>
         </is>
       </c>
       <c r="M1" s="5" t="inlineStr">
@@ -10335,13 +10335,13 @@
       <c r="E2" s="5" t="n">
         <v>500</v>
       </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="n">
+      <c r="F2" s="5" t="n">
         <v>0.12</v>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
       </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
@@ -10379,13 +10379,13 @@
       <c r="E3" s="5" t="n">
         <v>800</v>
       </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>2028</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="n">
+      <c r="F3" s="5" t="n">
         <v>0.12</v>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
@@ -10423,17 +10423,17 @@
       <c r="E4" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="n">
+      <c r="F4" s="5" t="n">
         <v>0.035</v>
       </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>floating</t>
+        </is>
+      </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>floating</t>
+          <t>cbr_key_rate</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
@@ -10471,17 +10471,17 @@
       <c r="E5" s="5" t="n">
         <v>1200</v>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>2028</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="n">
+      <c r="F5" s="5" t="n">
         <v>0.035</v>
       </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>floating</t>
+        </is>
+      </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>floating</t>
+          <t>cbr_key_rate</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
@@ -10519,13 +10519,13 @@
       <c r="E6" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>2027</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="n">
+      <c r="F6" s="5" t="n">
         <v>0.0575</v>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>floating</t>
+        </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
@@ -10563,13 +10563,13 @@
       <c r="E7" s="5" t="n">
         <v>1200</v>
       </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>2028</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="n">
+      <c r="F7" s="5" t="n">
         <v>0.07000000000000001</v>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
@@ -10607,13 +10607,13 @@
       <c r="E8" s="5" t="n">
         <v>800</v>
       </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>2027</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="n">
+      <c r="F8" s="5" t="n">
         <v>0.073</v>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>fixed</t>
+        </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
@@ -10651,17 +10651,17 @@
       <c r="E9" s="5" t="n">
         <v>1500</v>
       </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>2029</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="n">
+      <c r="F9" s="5" t="n">
         <v>0.02</v>
       </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>floating</t>
+        </is>
+      </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>floating</t>
+          <t>cbr_key_rate</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
@@ -10699,13 +10699,13 @@
       <c r="E10" s="5" t="n">
         <v>600</v>
       </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t>2028</t>
-        </is>
-      </c>
-      <c r="G10" s="5" t="n">
+      <c r="F10" s="5" t="n">
         <v>0.04</v>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>floating</t>
+        </is>
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
@@ -10743,17 +10743,17 @@
       <c r="E11" s="5" t="n">
         <v>96</v>
       </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="G11" s="5" t="n">
+      <c r="F11" s="5" t="n">
         <v>0.12</v>
       </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>floating</t>
+        </is>
+      </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>floating</t>
+          <t>cbr_key_rate</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">

</xml_diff>